<commit_message>
Scraping del 21/10 (ONPE, Estado, cursos) + respaldo datos.js para abrir la pagina en file://
</commit_message>
<xml_diff>
--- a/convocatorias.xlsx
+++ b/convocatorias.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -538,11 +538,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ONPE ERM-2026: ORIENTADORES CONV</t>
+          <t>ONPE ERM-2026: (06) AUXILIARES TÉCNICOS DIURNO DE ODPE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -552,27 +552,27 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Nivel Nacional</t>
+          <t>Requena, Huamalíes, Lima Oeste 1, Condesuyos, Mariscal Cáceres</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>S/. 1,800 Soles mensual (varia en proporción a los servicios prestados)</t>
+          <t>S/. 1800.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 433 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 17/09/2026 Vigente: Hasta el 27/09/2026, Según ODPE Salario: S/. 1,800 Soles mensual (varia en proporción a los servicios prestados) PUESTO: ORIENTADORES CONV NÚMERO: Locación de Servicios</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 6 Ubicación: Requena, Huamalíes, Lima Oeste 1, Condesuyos, Mariscal Cáceres Fecha de Publicación: 08/07/2026 Vigente: Hasta las 09:00 am. del 09/07/2026 Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO DIURNO DE ODPE NÚMERO: Locación de Servicios NIVEL:</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/09/onpe-erm-2026-orientadores-conv.html</t>
+          <t>https://www.portaltrabajos.pe/2026/07/onpe-erm-2026-06-auxiliares-tecnicos-diurno.html</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -592,12 +592,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1MeuPs3tLq2wAyDo-Zg5a0oBssgRbOVAT/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1UEMg-y-sQPh8rAi6f7S19fJ78Ga6FsUo/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1CE480QVirzMXLc_QqWPGZgS8JzmXhWgq/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/18jkuzD1VwyfhHf1sThllpzod4wIok7NA/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,21 +608,16 @@
       <c r="P2" t="inlineStr">
         <is>
           <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ONPE ERM-2026: AUXILIARES PARA REPLIEGUE DE ACTAS</t>
+          <t>ONPE ERM-2026: (125) AUXILIARES TÉCNICOS DIURNO DE ODPE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -637,22 +632,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>S/. 1,600 Soles mensual (varia en proporción a los servicios prestados)</t>
+          <t>S/. 1800.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 868 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 14/09/2026 Vigente: Hasta el 26/09/2026, Según ODPE Salario: S/. 1,600 Soles mensual (varia en proporción a los servicios prestados) PUESTO: AUXILIARES PARA REPLIEGUE DE ACTAS NÚMERO: Loca</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 125 Ubicación: Nivel Nacional Fecha de Publicación: 04/07/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO DIURNO DE ODPE NÚMERO: Locación de Servicios NIVEL: Secundaria Completa TIPO DE TRABAJO: Locaci</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/09/onpe-erm-2026-auxiliares-para-repliegue-actas.html</t>
+          <t>https://www.portaltrabajos.pe/2026/07/onpe-erm-2026-auxiliares-tecnicos-diurno-odpe.html</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -668,41 +663,16 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>si</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1g6J-FyYcTHU9XtL3sUgq--D_GEMvkFzc/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1_v5NI1v3YH-HqP7qzRInBQz98qc2WSY4/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ONPE ERM-2026: OPERADORES DE LA LINEA DE RECEPCIÓN</t>
+          <t>ONPE SEP-2026: ORIENTADORES CONV</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -717,22 +687,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>S/. 1,800 Soles mensual (varia en proporción a los servicios prestados)</t>
+          <t>S/. 420.00 Soles</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 224 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 14/09/2026 Vigente: Hasta el 28/09/2026, Según ODPE Salario: S/. 1,800 Soles mensual (varia en proporción a los servicios prestados) PUESTO: OPERADORES DE LA LINEA DE RECEPCIÓN NÚMERO: Loc</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 10,221 Ubicación: Nivel Nacional Fecha de Publicación: 25/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 420.00 Soles PUESTO: ORIENTADORES CONV NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE TRABAJO: Lo</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/09/onpe-erm-2026-operadores-de-la-linea-recepcion.html</t>
+          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-orientadores-conv.html</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -752,12 +722,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17koteXwoY6dV_9wCGNzpzjwVKzdc6QJM/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1NdtgUS0ZzEEt1vD_sQ-id4fZ1UqM7clS/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1wkqOJVwLCyhiygMjYHLAFkrw2OlFNret/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -768,21 +733,16 @@
       <c r="P4" t="inlineStr">
         <is>
           <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ONPE ERM-2026: RESPONSABLES DE LOCAL DE VOTACIÓN</t>
+          <t>ONPE SEP-2026: (304) RESPONSABLES DE LA LÍNEA DE RECEPCIÓN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -792,27 +752,27 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>HUAYTARA, ALTO AMAZONAS, HUANCAYO, HUAURA, MORROPON, LUCANAS</t>
+          <t>Nivel Nacional</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>S/. 2,500 Soles mensual (varia en proporción a los servicios prestados)</t>
+          <t>S/. 1,150.00 Soles</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 150 Ubicación: HUAYTARA, ALTO AMAZONAS, HUANCAYO, HUAURA, MORROPON, LUCANAS Fecha de Publicación: 29/08/2026 Vigente: Hasta el 27/09/2026, Según ODPE Salario: S/. 2,500 Soles mensual (varia en proporción a los servicios prestados) PUESTO: RESPONSABLES DE LOCAL DE VO</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 304 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Loca</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/08/onpe-erm-2026-responsables-de-local-de.html</t>
+          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-responsables-de-la-linea-recepcion.html</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -832,7 +792,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Jvtj7QBNaiPxcRQ5Dyywp5TmbPwcRn_Z/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1vGk0BVkB5XM6W8KFGXcotSYMtcTK_4Jp/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1zPTtsj0DRNCTzHYAUAurhXMo5nkHUoCP/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -843,21 +808,16 @@
       <c r="P5" t="inlineStr">
         <is>
           <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ONPE ERM-2026: COORDINADORES DE MESA</t>
+          <t>ONPE SEP-2026: (1,502) AUXILIARES DE CENTRO DE ACOPIO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -872,22 +832,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>S/. 2,000 Soles mensual (varia en proporción a los servicios prestados)</t>
+          <t>S/. 1,000 Soles</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2,312 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 22/08/2026 Vigente: Hasta el 27/09/2026, Según ODPE Salario: S/. 2,000 Soles mensual (varia en proporción a los servicios prestados) PUESTO: COORDINADORES DE MESA NÚMERO: Locación de Ser</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1,502 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,000 Soles PUESTO: AUXILIAR DE CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE TR</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/08/onpe-erm-2026-coordinadores-de-mesa.html</t>
+          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-auxiliares-de-centro-acopio.html</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -907,12 +867,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1fKWpUVW72Q2ZMgEIDQURmaEMylynFRwC/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1IQ7Utx9nyPPJFvhgJ422Gt-aNWaBaDkk/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ZueT04fQ3w8gEyzj-8drhLzh1TXHVxNm/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1PB5mND_4vyWHa8wKzezrJyyFNkzQQO8a/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -923,21 +883,16 @@
       <c r="P6" t="inlineStr">
         <is>
           <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ONPE ERM-2026: (06) AUXILIARES TÉCNICOS DIURNO DE ODPE</t>
+          <t>ONPE SEP-2026: (6,033) RESPONSABLES DE CENTRO DE ACOPIO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -947,27 +902,27 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Requena, Huamalíes, Lima Oeste 1, Condesuyos, Mariscal Cáceres</t>
+          <t>Nivel Nacional</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>S/. 1800.00 Soles mensuales</t>
+          <t>S/. 1,150.00 Soles</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 6 Ubicación: Requena, Huamalíes, Lima Oeste 1, Condesuyos, Mariscal Cáceres Fecha de Publicación: 08/07/2026 Vigente: Hasta las 09:00 am. del 09/07/2026 Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO DIURNO DE ODPE NÚMERO: Locación de Servicios NIVEL:</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 6,033 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Secundaria, Técnicos, Universitarios TIPO DE TRAB</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/07/onpe-erm-2026-06-auxiliares-tecnicos-diurno.html</t>
+          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-responsables-de-centro-acopio.html</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -987,12 +942,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1UEMg-y-sQPh8rAi6f7S19fJ78Ga6FsUo/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1wWZQJoLr-qxkxB5WKKjtKDlYsIBR3u-d/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/18jkuzD1VwyfhHf1sThllpzod4wIok7NA/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/18KMsQULKVem1ufZeOQcVty0XRveSfpGY/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1008,11 +963,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ONPE ERM-2026: (125) AUXILIARES TÉCNICOS DIURNO DE ODPE</t>
+          <t>ONPE SEP-2026: OPERADORES DE LA LÍNEA DE RECEPCIÓN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1027,22 +982,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>S/. 1800.00 Soles mensuales</t>
+          <t>S/. 900.00 Soles</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 125 Ubicación: Nivel Nacional Fecha de Publicación: 04/07/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO DIURNO DE ODPE NÚMERO: Locación de Servicios NIVEL: Secundaria Completa TIPO DE TRABAJO: Locaci</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2520 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 900.00 Soles PUESTO: OPERADORES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locació</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/07/onpe-erm-2026-auxiliares-tecnicos-diurno-odpe.html</t>
+          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-operadores-de-linea-recepcion.html</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1058,16 +1013,36 @@
       <c r="L8" t="inlineStr">
         <is>
           <t>si</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/13qDCjyDgy0BFynlfrXhfYORlEqeAcbbs/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1ru-5Z0loVFuLOS9e2pz3J8xDU_-1uQkk/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ONPE SEP-2026: ORIENTADORES CONV</t>
+          <t>ONPE SEP-2026: (7,461) AUXILIARES PARA REPLIEGUE DE ACTAS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1082,22 +1057,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>S/. 420.00 Soles</t>
+          <t>S/. 800.00 Soles</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 10,221 Ubicación: Nivel Nacional Fecha de Publicación: 25/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 420.00 Soles PUESTO: ORIENTADORES CONV NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE TRABAJO: Lo</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 7,461 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 800.00 Soles PUESTO: AUXILIARES PARA REPLIEGUE DE ACTAS NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIP</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-orientadores-conv.html</t>
+          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-auxiliares-para-repliegue-actas.html</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1117,7 +1092,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1wkqOJVwLCyhiygMjYHLAFkrw2OlFNret/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1MfRsOF5WEjaBcaJd9L31U34JVOukjutO/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1XiisjecZvd9xBhJkcsHkEyBfoYDgKNA1/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1133,11 +1113,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ONPE SEP-2026: (304) RESPONSABLES DE LA LÍNEA DE RECEPCIÓN</t>
+          <t>ONPE SEP-2026: (10) ANALISTAS DESCENTRALIZADOS DE RECURSOS HUMANOS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1147,27 +1127,27 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nivel Nacional</t>
+          <t>ODPE DE PROVINCIAS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>S/. 1,150.00 Soles</t>
+          <t>Entre S/ 5,000 a S/ 6,000 soles</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 304 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Loca</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 10 Ubicación: ODPE DE PROVINCIAS Fecha de Publicación: 21/04/2026 Vigente: Hasta completar vacantes, según ODPE Salario: Entre S/ 5,000 a S/ 6,000 soles PUESTO: ANALISTAS DESCENTRALIZADOS DE RECURSOS HUMANOS - ACTUALIZACIÓN DE BASE DE DATOS NÚMERO: Locación de Servi</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-responsables-de-la-linea-recepcion.html</t>
+          <t>https://www.portaltrabajos.pe/2026/04/onpe-sep-2026-analistas-descentralizados.html</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1187,12 +1167,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1vGk0BVkB5XM6W8KFGXcotSYMtcTK_4Jp/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1zPTtsj0DRNCTzHYAUAurhXMo5nkHUoCP/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/14y8lKpt1-ALev_QfHRfrsypVpokvPtQX/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1208,11 +1183,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ONPE SEP-2026: (1,502) AUXILIARES DE CENTRO DE ACOPIO</t>
+          <t>ONPE EG2026: (2,603) AUXILIARES PARA REPLIEGUE DE ACTAS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1227,22 +1202,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>S/. 1,000 Soles</t>
+          <t>S/. 800.00 Soles</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1,502 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,000 Soles PUESTO: AUXILIAR DE CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE TR</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2,603 Ubicación: Nivel Nacional Fecha de Publicación: 24/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 800.00 Soles PUESTO: AUXILIARES PARA REPLIEGUE DE ACTAS NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIP</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-auxiliares-de-centro-acopio.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-para-repliegue-actas.html</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1262,12 +1237,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1IQ7Utx9nyPPJFvhgJ422Gt-aNWaBaDkk/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1ov-cSSt2rOgD8sYdehoJVOx4KSnjC798/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1PB5mND_4vyWHa8wKzezrJyyFNkzQQO8a/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1XiisjecZvd9xBhJkcsHkEyBfoYDgKNA1/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1283,11 +1258,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ONPE SEP-2026: (6,033) RESPONSABLES DE CENTRO DE ACOPIO</t>
+          <t>ONPE EG2026: (1,358) AUXILIARES DEL CENTRO DE ACOPIO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1302,22 +1277,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>S/. 1,150.00 Soles</t>
+          <t>S/. 933.33 Soles</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 6,033 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Secundaria, Técnicos, Universitarios TIPO DE TRAB</t>
+          <t xml:space="preserve">Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1,358 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 933.33 Soles PUESTO: AUXILIAR DEL CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE </t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-responsables-de-centro-acopio.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-del-centro-acopio.html</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1337,12 +1312,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1wWZQJoLr-qxkxB5WKKjtKDlYsIBR3u-d/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1pxMIgAZWBp8s9sN5zE8_NS_hsTbWGoPE/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/18KMsQULKVem1ufZeOQcVty0XRveSfpGY/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1PB5mND_4vyWHa8wKzezrJyyFNkzQQO8a/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1358,11 +1333,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ONPE SEP-2026: OPERADORES DE LA LÍNEA DE RECEPCIÓN</t>
+          <t>ONPE EG2026: (2,307) AUXILIARES TÉCNICOS DE LOCAL DE VOTACION</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1372,27 +1347,27 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nivel Nacional</t>
+          <t>Lima, Callao</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>S/. 900.00 Soles</t>
+          <t>S/. 1,000.00 Soles</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2520 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 900.00 Soles PUESTO: OPERADORES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locació</t>
+          <t xml:space="preserve">Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2,307 Ubicación: Lima, Callao Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,000.00 Soles PUESTO: AUXILIAR TÉCNICO DE LOCAL DE VOTACIÓN NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios </t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-operadores-de-linea-recepcion.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-tecnicos-de-local-de-votacion.html</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1408,36 +1383,16 @@
       <c r="L13" t="inlineStr">
         <is>
           <t>si</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/13qDCjyDgy0BFynlfrXhfYORlEqeAcbbs/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1ru-5Z0loVFuLOS9e2pz3J8xDU_-1uQkk/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ONPE SEP-2026: (7,461) AUXILIARES PARA REPLIEGUE DE ACTAS</t>
+          <t>ONPE EG2026: (5,675) RESPONSABLES DE CENTRO DE ACOPIO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1452,22 +1407,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>S/. 800.00 Soles</t>
+          <t>S/. 1,150.00 Soles</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 7,461 Ubicación: Nivel Nacional Fecha de Publicación: 18/05/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 800.00 Soles PUESTO: AUXILIARES PARA REPLIEGUE DE ACTAS NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIP</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 5,675 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locació</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/05/onpe-sep-2026-auxiliares-para-repliegue-actas.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-responsables-de-centro-de-acopio.html</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1487,12 +1442,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1MfRsOF5WEjaBcaJd9L31U34JVOukjutO/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1SvDeSxFdMaik3MQYhHVlKYcKQFPCc3gS/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1XiisjecZvd9xBhJkcsHkEyBfoYDgKNA1/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/18KMsQULKVem1ufZeOQcVty0XRveSfpGY/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1508,11 +1463,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ONPE SEP-2026: (10) ANALISTAS DESCENTRALIZADOS DE RECURSOS HUMANOS</t>
+          <t>ONPE EG2026: (2,440) OPERADORES DE LA LÍNEA DE RECEPCIÓN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1522,27 +1477,27 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ODPE DE PROVINCIAS</t>
+          <t>Nivel Nacional</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Entre S/ 5,000 a S/ 6,000 soles</t>
+          <t>S/. 900.00 Soles</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 10 Ubicación: ODPE DE PROVINCIAS Fecha de Publicación: 21/04/2026 Vigente: Hasta completar vacantes, según ODPE Salario: Entre S/ 5,000 a S/ 6,000 soles PUESTO: ANALISTAS DESCENTRALIZADOS DE RECURSOS HUMANOS - ACTUALIZACIÓN DE BASE DE DATOS NÚMERO: Locación de Servi</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2440 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 900.00 Soles PUESTO: OPERADORES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locació</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/04/onpe-sep-2026-analistas-descentralizados.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-operadores-de-la-line.html</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1562,7 +1517,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/14y8lKpt1-ALev_QfHRfrsypVpokvPtQX/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1FyzjGwERlrUBv3CFk-bTSrHrRev61kZw/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1ru-5Z0loVFuLOS9e2pz3J8xDU_-1uQkk/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1578,11 +1538,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (2,603) AUXILIARES PARA REPLIEGUE DE ACTAS</t>
+          <t>ONPE EG2026: (306) RESPONSABLES DE LA LÍNEA DE RECEPCIÓN</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1597,22 +1557,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>S/. 800.00 Soles</t>
+          <t>S/. 1,150.00 Soles</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2,603 Ubicación: Nivel Nacional Fecha de Publicación: 24/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 800.00 Soles PUESTO: AUXILIARES PARA REPLIEGUE DE ACTAS NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIP</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 306 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Loca</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-para-repliegue-actas.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-responsables-de-la-linea-recepcion.html</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1632,12 +1592,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ov-cSSt2rOgD8sYdehoJVOx4KSnjC798/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/15WCj6VEV3iECe4I1nQ9j173N6z1dylHG/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1XiisjecZvd9xBhJkcsHkEyBfoYDgKNA1/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1zPTtsj0DRNCTzHYAUAurhXMo5nkHUoCP/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1653,11 +1613,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (1,358) AUXILIARES DEL CENTRO DE ACOPIO</t>
+          <t>ONPE EG2026: (10,334) ORIENTADORES CONV/STAE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1672,17 +1632,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>S/. 933.33 Soles</t>
+          <t>S/. 420.00 Soles</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1,358 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 933.33 Soles PUESTO: AUXILIAR DEL CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE </t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 10334 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 420.00 Soles PUESTO: ORIENTADORES CONV/STAE NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE TRABAJO</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-del-centro-acopio.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-orientadores-conv-stae..html</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1707,12 +1667,12 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pxMIgAZWBp8s9sN5zE8_NS_hsTbWGoPE/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1Lu9O7UmGqk46NpAJUhJGSD_EvrJKZHhd/view?usp=drive_link</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1PB5mND_4vyWHa8wKzezrJyyFNkzQQO8a/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1C_2-4BXAzxMsV1or_kRUhG7EE_hva3Iq/view?usp=drive_link</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1728,11 +1688,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (2,307) AUXILIARES TÉCNICOS DE LOCAL DE VOTACION</t>
+          <t>ONPE EG2026: (2307) TÉCNICOS DE TRANSMISIÓN DE LOCAL DE VOTACIÓN</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1742,27 +1702,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Lima, Callao</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>S/. 1,000.00 Soles</t>
+          <t>S/. 1,000.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2,307 Ubicación: Lima, Callao Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,000.00 Soles PUESTO: AUXILIAR TÉCNICO DE LOCAL DE VOTACIÓN NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios </t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2307 Ubicación: Lima Fecha de Publicación: 20/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,000.00 Soles mensuales PUESTO: TÉCNICO DE TRANSMISIÓN DE LOCAL DE VOTACIÓN NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universi</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-tecnicos-de-local-de-votacion.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-tecnicos-de-transmision.html</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1778,16 +1738,36 @@
       <c r="L18" t="inlineStr">
         <is>
           <t>si</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1xIA11au143GKiuiLOYRcEupHijoClntD/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1Rqzwmrn7Hd1gmpuheI4ayk-kR9coW-zX/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (5,675) RESPONSABLES DE CENTRO DE ACOPIO</t>
+          <t>ONPE EG2026: (278) AUXILIARES ADMINISTRATIVOS T2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1802,22 +1782,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>S/. 1,150.00 Soles</t>
+          <t>S/. 2200.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 5,675 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE CENTRO DE ACOPIO NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locació</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 278 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 03/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES ADMINISTRATIVOS T2 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universit</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-responsables-de-centro-de-acopio.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-administrativos-t2.html</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1837,12 +1817,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1SvDeSxFdMaik3MQYhHVlKYcKQFPCc3gS/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_ADMINISTRATIVO_T2.pdf</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/18KMsQULKVem1ufZeOQcVty0XRveSfpGY/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_ADMINISTRATIVO_T2.pdf</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1858,11 +1838,11 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (2,440) OPERADORES DE LA LÍNEA DE RECEPCIÓN</t>
+          <t>ONPE EG2026: (280) AUXILIARES DE OPERACIONES T2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1877,22 +1857,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>S/. 900.00 Soles</t>
+          <t>S/. 2200.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2440 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 900.00 Soles PUESTO: OPERADORES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locació</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 280 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 03/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DE OPERACIONES T2 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universita</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-operadores-de-la-line.html</t>
+          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-de-operaciones-t2.html</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1912,12 +1892,12 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FyzjGwERlrUBv3CFk-bTSrHrRev61kZw/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR-DE-OPERACIONES-T2.pdf</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ru-5Z0loVFuLOS9e2pz3J8xDU_-1uQkk/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES-AUXILIAR-DE-OPERACIONES-T2.pdf</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1933,11 +1913,11 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (306) RESPONSABLES DE LA LÍNEA DE RECEPCIÓN</t>
+          <t>ONPE EG2026: (7,681) RESPONSABLES DE LOCAL DE VOTACIÓN</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1952,22 +1932,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>S/. 1,150.00 Soles</t>
+          <t>S/. 2500.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 306 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,150.00 Soles PUESTO: RESPONSABLES DE LA LÍNEA DE RECEPCIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Loca</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 7,681 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 26/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2500.00 Soles mensuales PUESTO: RESPONSABLE DE LOCAL DE VOTACIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Univ</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-responsables-de-la-linea-recepcion.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-responsables-de-local-de-votacion.html</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1987,12 +1967,12 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15WCj6VEV3iECe4I1nQ9j173N6z1dylHG/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/RESPONSABLE_DE_LOCAL_DE_VOTACION.pdf</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1zPTtsj0DRNCTzHYAUAurhXMo5nkHUoCP/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_RESPONSABLE_DE_LOCAL_DE_VOTACION.pdf</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2008,11 +1988,11 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (10,334) ORIENTADORES CONV/STAE</t>
+          <t>ONPE: (15) SOPORTE DE CONSULADO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2022,27 +2002,27 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Nivel Nacional</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>S/. 420.00 Soles</t>
+          <t>S/. 2,000.00 Soles</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 10334 Ubicación: Nivel Nacional Fecha de Publicación: 21/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 420.00 Soles PUESTO: ORIENTADORES CONV/STAE NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universitarios TIPO DE TRABAJO</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 15 Ubicación: Lima Fecha de Publicación: 24/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2,000.00 Soles PUESTO: SOPORTE DE CONSULADO NÚMERO: Locación de Servicios NIVEL: Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Presencia</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-orientadores-conv-stae..html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-soporte-de-consulado.html</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2062,17 +2042,17 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Lu9O7UmGqk46NpAJUhJGSD_EvrJKZHhd/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/SOPORTE_DE_CONSULADO.pdf</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1C_2-4BXAzxMsV1or_kRUhG7EE_hva3Iq/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_SOPORTE_DE_CONSULADO.pdf</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
+          <t>https://www.onpe.gob.pe/modTransparencia/Convocatorias/LOC/Guia-Postulante-Educate-onpev3.pdf</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2083,11 +2063,11 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (2307) TÉCNICOS DE TRANSMISIÓN DE LOCAL DE VOTACIÓN</t>
+          <t>ONPE EG2026: (5,675) RESPONSABLES DE CENTRO DE ACOPIO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2097,27 +2077,27 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Nivel Nacional</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>S/. 1,000.00 Soles mensuales</t>
+          <t>S/. 2300.00 Soles</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 2307 Ubicación: Lima Fecha de Publicación: 20/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1,000.00 Soles mensuales PUESTO: TÉCNICO DE TRANSMISIÓN DE LOCAL DE VOTACIÓN NÚMERO: Locación de Servicios NIVEL: Secundaria Completa, Técnicos, Universi</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 5,675 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 23/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2300.00 Soles PUESTO: COORDINADOR DE MESA NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRAB</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-tecnicos-de-transmision.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-responsables-de-centro-acopio.html</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2137,12 +2117,12 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1xIA11au143GKiuiLOYRcEupHijoClntD/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/RESPONSABLE_DE_CENTRO_DE_ACOPIO.pdf</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Rqzwmrn7Hd1gmpuheI4ayk-kR9coW-zX/view?usp=drive_link</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_RESPONSABLE_DE_CENTRO_DE_ACOPIO.pdf</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2158,11 +2138,11 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (278) AUXILIARES ADMINISTRATIVOS T2</t>
+          <t>ONPE EG2026: (23,192) COORDINADORES DE MESA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2177,22 +2157,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>S/. 2200.00 Soles mensuales</t>
+          <t>S/. 2000.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 278 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 03/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES ADMINISTRATIVOS T2 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universit</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 23,192 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 23/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2000.00 Soles mensuales PUESTO: COORDINADOR DE MESA NÚMERO: Locación de Servicios NIVEL: Secundaria, Técnicos, Univ</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-administrativos-t2.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-coordinadores-de-mesa.html</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2208,36 +2188,16 @@
       <c r="L24" t="inlineStr">
         <is>
           <t>si</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_ADMINISTRATIVO_T2.pdf</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_ADMINISTRATIVO_T2.pdf</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (280) AUXILIARES DE OPERACIONES T2</t>
+          <t>ONPE EG2026: (198) AUXILIARES DEL CENTRO DE CÓMPUTO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2257,17 +2217,17 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 280 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 03/03/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DE OPERACIONES T2 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universita</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 198 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 20/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DEL CENTRO DE CÓMPUTO NÚMERO: Locación de Servicios NIVEL: Técnicos, Univer</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/03/onpe-eg2026-auxiliares-de-operaciones-t2.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliares-del-centro-computo.html</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2287,12 +2247,12 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR-DE-OPERACIONES-T2.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_DEL_CENTRO_DE_COMPUTO.pdf</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES-AUXILIAR-DE-OPERACIONES-T2.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_DEL_CENTRO_DE_COMPUTO.pdf</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2308,11 +2268,11 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (7,681) RESPONSABLES DE LOCAL DE VOTACIÓN</t>
+          <t>ONPE EG2026: (4230) OPERADORES DEL CENTRO DE CÓMPUTO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2327,22 +2287,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>S/. 2500.00 Soles mensuales</t>
+          <t>S/. 1800.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 7,681 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 26/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2500.00 Soles mensuales PUESTO: RESPONSABLE DE LOCAL DE VOTACIÓN NÚMERO: Locación de Servicios NIVEL: Técnicos, Univ</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 4230 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 20/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: OPERADORES DEL CENTRO DE CÓMPUTO NÚMERO: Locación de Servicios NIVEL: Secundaria, Téc</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-responsables-de-local-de-votacion.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-operadores-del-centro-de-computo.html</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2362,12 +2322,12 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/RESPONSABLE_DE_LOCAL_DE_VOTACION.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/OPERADORES_DEL_CENTRO_DE_COMPUTO.pdf</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_RESPONSABLE_DE_LOCAL_DE_VOTACION.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_OPERADORES_DEL_CENTRO_DE_COMPUTO.pdf</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2383,11 +2343,11 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ONPE: (15) SOPORTE DE CONSULADO</t>
+          <t>ONPE: (15,044) COORDINADORES TÉCNICOS DE MESA STAE</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2397,27 +2357,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Callao, Lima</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>S/. 2,000.00 Soles</t>
+          <t>S/. 2000.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 15 Ubicación: Lima Fecha de Publicación: 24/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2,000.00 Soles PUESTO: SOPORTE DE CONSULADO NÚMERO: Locación de Servicios NIVEL: Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Presencia</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 15,044 Ubicación: Callao, Lima Fecha de Publicación: 09/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2000.00 Soles mensuales PUESTO: COORDINADORES TÉCNICOS DE MESA STAE NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABA</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-soporte-de-consulado.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-coordinadores-tecnicos-de-mesa-stae.html</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2437,12 +2397,12 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/SOPORTE_DE_CONSULADO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/COORDINADOR_TECNICO_MESA_STAE_03_03_2026.pdf</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_SOPORTE_DE_CONSULADO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES-COORDINADORES-TECNICOS-DE-MESA-STAE.pdf</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2458,11 +2418,11 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (5,675) RESPONSABLES DE CENTRO DE ACOPIO</t>
+          <t>ONPE: (4,093) CAPACITADORES CONVENCIONAL/STAE/ CCPP</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2477,22 +2437,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>S/. 2300.00 Soles</t>
+          <t>S/. 2800.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 5,675 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 23/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2300.00 Soles PUESTO: COORDINADOR DE MESA NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRAB</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 4,093 Ubicación: Nivel Nacional Fecha de Publicación: 09/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2800.00 Soles mensuales PUESTO: CAPACITADORES CONVENCIONAL/STAE/ CCPP NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TR</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-responsables-de-centro-acopio.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-capacitadores-convencional.html</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2512,17 +2472,17 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/RESPONSABLE_DE_CENTRO_DE_ACOPIO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/CAPACITADORES_STAE_CCPP.pdf</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_RESPONSABLE_DE_CENTRO_DE_ACOPIO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_CAPACITADORES_STAE_CCPP.pdf</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
+          <t>https://www.onpe.gob.pe/modTransparencia/Convocatorias/LOC/Guia-Postulante-Educate-onpev3.pdf</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -2533,11 +2493,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (23,192) COORDINADORES DE MESA</t>
+          <t>ONPE EG2026: (213) AUXILIARES TÉCNICOS NOCTURNO DISTRITAL STAE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2547,27 +2507,27 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Nivel Nacional</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>S/. 2000.00 Soles mensuales</t>
+          <t>S/. 1800.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 23,192 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 23/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2000.00 Soles mensuales PUESTO: COORDINADOR DE MESA NÚMERO: Locación de Servicios NIVEL: Secundaria, Técnicos, Univ</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 213 Ubicación: Lima - (Según ODPE Disponible) Fecha de Publicación: 16/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO NOCTURNO DISTRITAL STAE NÚMERO: Locación de Servicios NIVEL: Secundaria Complet</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-coordinadores-de-mesa.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliares-tecnicos-nocturno-distrital.html</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2583,16 +2543,36 @@
       <c r="L29" t="inlineStr">
         <is>
           <t>si</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_TECNICO_NOCTURNO_DISTRITAL_STAE.pdf</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_TECNICO_NOCTURNO_DISTRITAL_STAE.pdf</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (198) AUXILIARES DEL CENTRO DE CÓMPUTO</t>
+          <t>ONPE EG2026: (213) AUXILIARES TÉCNICOS DIURNO DISTRITAL STAE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2602,27 +2582,27 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Nivel Nacional</t>
+          <t>Lima</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>S/. 2200.00 Soles mensuales</t>
+          <t>S/. 1800.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 198 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 20/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DEL CENTRO DE CÓMPUTO NÚMERO: Locación de Servicios NIVEL: Técnicos, Univer</t>
+          <t xml:space="preserve">Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 213 Ubicación: Lima - (Según ODPE Disponible) Fecha de Publicación: 16/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO DIURNO DISTRITAL STAE NÚMERO: Locación de Servicios NIVEL: Secundaria Completa </t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliares-del-centro-computo.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliar-tecnico-diurno-distrital-stae.html</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2642,12 +2622,12 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_DEL_CENTRO_DE_COMPUTO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_TECNICO_DIURNO_DISTRITAL_STAE.pdf</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_DEL_CENTRO_DE_COMPUTO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_TECNICO_DIURNO_DISTRITAL_STAE.pdf</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2663,11 +2643,11 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (4230) OPERADORES DEL CENTRO DE CÓMPUTO</t>
+          <t>ONPE EG2026: (483) AUXILIARES DE RECURSOS HUMANOS T2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2682,22 +2662,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>S/. 1800.00 Soles mensuales</t>
+          <t>S/. 2200.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 4230 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 20/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: OPERADORES DEL CENTRO DE CÓMPUTO NÚMERO: Locación de Servicios NIVEL: Secundaria, Téc</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 483 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 16/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DE OPERACIONES T1 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universita</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-operadores-del-centro-de-computo.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliar-de-recursos-humanos.html</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2717,12 +2697,12 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/OPERADORES_DEL_CENTRO_DE_COMPUTO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_DE_RECURSOS_HUMANOS_T2.pdf</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_OPERADORES_DEL_CENTRO_DE_COMPUTO.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_DE_RECURSOS_HUMANOS_T2.pdf</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2738,11 +2718,11 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ONPE: (15,044) COORDINADORES TÉCNICOS DE MESA STAE</t>
+          <t>¡ATENCIÓN! ONPE lanzará convocatoria para más de 21,000 Coordinadores de Mesa a nivel nacional</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2750,29 +2730,19 @@
           <t>ONPE</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Callao, Lima</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>S/. 2000.00 Soles mensuales</t>
-        </is>
-      </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 15,044 Ubicación: Callao, Lima Fecha de Publicación: 09/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2000.00 Soles mensuales PUESTO: COORDINADORES TÉCNICOS DE MESA STAE NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABA</t>
+          <t>Si estás buscando una oportunidad laboral para este 2026, ¡esta es tu oportunidad! En el marco de las próximas Elecciones Generales 2026 , la Oficina Nacional de Procesos Electorales (ONPE) tiene previsto lanzar una de sus convocatorias más grandes para el puesto de Coordinador de Mesa a nivel nacional. Detalles de la convocator</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-coordinadores-tecnicos-de-mesa-stae.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-lanzara-convocatoria-para-mas-de-21000-coordinadores-de-mesa.html</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2787,37 +2757,17 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/COORDINADOR_TECNICO_MESA_STAE_03_03_2026.pdf</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES-COORDINADORES-TECNICOS-DE-MESA-STAE.pdf</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>https://www.onpe.gob.pe/modTransparencia/Convocatorias/LOC/Guia-Postulante-Educate-onpev3.pdf</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ONPE: (4,093) CAPACITADORES CONVENCIONAL/STAE/ CCPP</t>
+          <t>ONPE: ¿Cuáles son las Funciones de los Coordinadores Técnicos de Mesa STAE? - EG2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2825,29 +2775,19 @@
           <t>ONPE</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Nivel Nacional</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>S/. 2800.00 Soles mensuales</t>
-        </is>
-      </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 4,093 Ubicación: Nivel Nacional Fecha de Publicación: 09/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2800.00 Soles mensuales PUESTO: CAPACITADORES CONVENCIONAL/STAE/ CCPP NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TR</t>
+          <t>El 12 de Abril de 2026, se llevará a cabo las Elecciones Generales 2026 , en ese sentido la ONPE ha lanzado la convocatoria para cubrir más de 15,000 plazas de Coordinadores Técnicos de Mesa STAE para Lima y Callao. En todo Lima Metropolitana y el Callao, los miembros de mesa harán uso de la Solución Tecnológica de Apoyo al Escr</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-capacitadores-convencional.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-cuales-son-las-funciones-de-los-coordinadores-tecnicos-de-mesa-stae.html</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2862,37 +2802,17 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/CAPACITADORES_STAE_CCPP.pdf</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_CAPACITADORES_STAE_CCPP.pdf</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>https://www.onpe.gob.pe/modTransparencia/Convocatorias/LOC/Guia-Postulante-Educate-onpev3.pdf</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (213) AUXILIARES TÉCNICOS NOCTURNO DISTRITAL STAE</t>
+          <t>ONPE EG2026: (407) AUXILIARES DE OPERACIONES T1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2902,27 +2822,27 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Nivel Nacional</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>S/. 1800.00 Soles mensuales</t>
+          <t>S/. 2200.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 213 Ubicación: Lima - (Según ODPE Disponible) Fecha de Publicación: 16/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO NOCTURNO DISTRITAL STAE NÚMERO: Locación de Servicios NIVEL: Secundaria Complet</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 407 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 12/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DE OPERACIONES T1 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universita</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliares-tecnicos-nocturno-distrital.html</t>
+          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-auxiliares-de-operaciones.html</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2942,12 +2862,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_TECNICO_NOCTURNO_DISTRITAL_STAE.pdf</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_TECNICO_NOCTURNO_DISTRITAL_STAE.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_DE_OPERACIONES_T1.pdf</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2963,11 +2878,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (213) AUXILIARES TÉCNICOS DIURNO DISTRITAL STAE</t>
+          <t>ONPE - EG2026: ¿Cuáles son las Funciones de los Coordinadores de Local de Votación?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2975,29 +2890,19 @@
           <t>ONPE</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Lima</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>S/. 1800.00 Soles mensuales</t>
-        </is>
-      </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 213 Ubicación: Lima - (Según ODPE Disponible) Fecha de Publicación: 16/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 1800.00 Soles mensuales PUESTO: AUXILIAR TÉCNICO DIURNO DISTRITAL STAE NÚMERO: Locación de Servicios NIVEL: Secundaria Completa </t>
+          <t>Con miras a las próximas Elecciones Generales 2026 , donde los peruanos elegiremos al próximo Presidente, Vicepresidentes, Diputados, Senadores y representantes ante el Parlamento Andino, la ONPE ha lanzado la convocatoria oficial para cubrir las plazas de Coordinadores de Local de Votación (CLV) a nivel nacional. Ante la magnit</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliar-tecnico-diurno-distrital-stae.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-cuales-son-las-funciones-de-los-CLV.html</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3012,37 +2917,17 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_TECNICO_DIURNO_DISTRITAL_STAE.pdf</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_TECNICO_DIURNO_DISTRITAL_STAE.pdf</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (483) AUXILIARES DE RECURSOS HUMANOS T2</t>
+          <t>¡PRÓXIMAMENTE! ONPE LANZARÁ MÁS DE 60,000 PLAZAS, PARA LAS ELECCIONES GENERALES 2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3050,29 +2935,19 @@
           <t>ONPE</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Nivel Nacional</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>S/. 2200.00 Soles mensuales</t>
-        </is>
-      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 483 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 16/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DE OPERACIONES T1 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universita</t>
+          <t>La Oficina Nacional de Procesos Electorales (ONPE), iniciará próximamente la contratación masiva de personal a nivel nacional. Conoce los perfiles, sueldos y fechas clave para postular. El organismo electoral se prepara para el despliegue logístico más grande del país. Ante la proximidad de las Elecciones Generales 2026, se ha c</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-auxiliar-de-recursos-humanos.html</t>
+          <t>https://www.portaltrabajos.pe/2026/02/proximamente-onpe-lanzara-mas-de-60000-plazas-eg2026.html</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3087,37 +2962,17 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_DE_RECURSOS_HUMANOS_T2.pdf</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_AUXILIAR_DE_RECURSOS_HUMANOS_T2.pdf</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>¡ATENCIÓN! ONPE lanzará convocatoria para más de 21,000 Coordinadores de Mesa a nivel nacional</t>
+          <t>ONPE EG2026: Asistentes de Oficina T2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3125,19 +2980,29 @@
           <t>ONPE</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Nivel Nacional</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>S/. 2500.00 Soles mensuales</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Si estás buscando una oportunidad laboral para este 2026, ¡esta es tu oportunidad! En el marco de las próximas Elecciones Generales 2026 , la Oficina Nacional de Procesos Electorales (ONPE) tiene previsto lanzar una de sus convocatorias más grandes para el puesto de Coordinador de Mesa a nivel nacional. Detalles de la convocator</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 282 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 30/01/2026 Vigente: Según ODPE Salario: S/. 2500.00 Soles mensuales PUESTO: ASISTENTES DE OFICINA NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locación de</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-lanzara-convocatoria-para-mas-de-21000-coordinadores-de-mesa.html</t>
+          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-asistentes-de-oficina-t2.html</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3152,17 +3017,32 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/ASISTENTE_DE_OFICINA_T2.pdf</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/GUIA_PARA_POSTULAR_ONPE.pdf</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ONPE: ¿Cuáles son las Funciones de los Coordinadores Técnicos de Mesa STAE? - EG2026</t>
+          <t>ONPE - CONSULTA SI ERES MIEMBRO DE MESA - ELECCIONES GENERALES 2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3172,17 +3052,17 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>El 12 de Abril de 2026, se llevará a cabo las Elecciones Generales 2026 , en ese sentido la ONPE ha lanzado la convocatoria para cubrir más de 15,000 plazas de Coordinadores Técnicos de Mesa STAE para Lima y Callao. En todo Lima Metropolitana y el Callao, los miembros de mesa harán uso de la Solución Tecnológica de Apoyo al Escr</t>
+          <t>El 12 de abril del 2026, es el día de las Elecciones Generales 2026, en ese sentido si deseas conocer si eres miembro de mesa, te informamos que la ONPE ya publicó el link donde puedes CONSULTAR SI ERES MIEMBRO DE MESA , para las Elecciones Generales 2026. Ingresa en el siguiente link para consultar si eres miembro de mesa: http</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-cuales-son-las-funciones-de-los-coordinadores-tecnicos-de-mesa-stae.html</t>
+          <t>https://www.portaltrabajos.pe/2026/01/onpe-consulta-si-eres-miembro-de-mesa.html</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3203,11 +3083,11 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ONPE EG2026: (407) AUXILIARES DE OPERACIONES T1</t>
+          <t>ONPE EG2026: Asistentes Legales</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3222,22 +3102,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>S/. 2200.00 Soles mensuales</t>
+          <t>S/. 4000.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 407 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 12/02/2026 Vigente: Hasta completar vacantes, según ODPE Salario: S/. 2200.00 Soles mensuales PUESTO: AUXILIARES DE OPERACIONES T1 NÚMERO: Locación de Servicios NIVEL: Técnicos, Universita</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 126 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 27/01/2026 Vigente: Según ODPE Salario: S/. 4000.00 Soles mensuales PUESTO: ASISTENTES LEGALES NÚMERO: Locación de Servicios NIVEL: Universitarios TIPO DE TRABAJO: Locación de Servicios MO</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-auxiliares-de-operaciones.html</t>
+          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-asistentes-legales.html</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3257,7 +3137,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/AUXILIAR_DE_OPERACIONES_T1.pdf</t>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/ASISTENTE_LEGAL.pdf</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -3273,11 +3153,11 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ONPE - EG2026: ¿Cuáles son las Funciones de los Coordinadores de Local de Votación?</t>
+          <t>ONPE EG2026: (1895) Coordinadores de Centro Poblado</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3285,19 +3165,29 @@
           <t>ONPE</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Nivel Nacional</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>S/. 3000.00 Soles mensuales</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Con miras a las próximas Elecciones Generales 2026 , donde los peruanos elegiremos al próximo Presidente, Vicepresidentes, Diputados, Senadores y representantes ante el Parlamento Andino, la ONPE ha lanzado la convocatoria oficial para cubrir las plazas de Coordinadores de Local de Votación (CLV) a nivel nacional. Ante la magnit</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1895 Ubicación: Nivel Nacional Fecha de Publicación: 24/01/2026 Vigente: Según ODPE Salario: S/. 3000.00 Soles mensuales PUESTO: COORDINADOR DISTRITAL NÚMERO: Locación de Servicios NIVEL: Técnicos y Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Pr</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/onpe-eg2026-cuales-son-las-funciones-de-los-CLV.html</t>
+          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-coordinadores-de-centro-poblado.html</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3312,17 +3202,32 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/COORDINADOR_DE_CENTRO_%20POBLADO_ODPE_EG2026.pdf</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>¡PRÓXIMAMENTE! ONPE LANZARÁ MÁS DE 60,000 PLAZAS, PARA LAS ELECCIONES GENERALES 2026</t>
+          <t>ONPE EG2026: (203) Coordinadores Distritales STAE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3330,19 +3235,29 @@
           <t>ONPE</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Lima</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>S/. 3000.00 Soles mensuales</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>La Oficina Nacional de Procesos Electorales (ONPE), iniciará próximamente la contratación masiva de personal a nivel nacional. Conoce los perfiles, sueldos y fechas clave para postular. El organismo electoral se prepara para el despliegue logístico más grande del país. Ante la proximidad de las Elecciones Generales 2026, se ha c</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 203 Ubicación: Lima Fecha de Publicación: 15/02/2026 Vigente: Según ODPE Salario: S/. 3000.00 Soles mensuales PUESTO: COORDINADOR DISTRITAL STAE NÚMERO: Locación de Servicios NIVEL: Técnicos y Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Presenci</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/02/proximamente-onpe-lanzara-mas-de-60000-plazas-eg2026.html</t>
+          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-coordinadores-stae.html</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3357,17 +3272,37 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/COORDINADOR_DISTRITAL_ODPE_STAE_EG2026.pdf</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_COORDINADORES_DISTRITALES_STAE.pdf</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>https://reclutamiento.onpe.gob.pe/login</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ONPE EG2026: Asistentes de Oficina T2</t>
+          <t>ONPE EG2026: (1990) Coordinadores Distritales</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3382,22 +3317,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>S/. 2500.00 Soles mensuales</t>
+          <t>S/. 3000.00 Soles mensuales</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 282 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 30/01/2026 Vigente: Según ODPE Salario: S/. 2500.00 Soles mensuales PUESTO: ASISTENTES DE OFICINA NÚMERO: Locación de Servicios NIVEL: Técnicos, Universitarios TIPO DE TRABAJO: Locación de</t>
+          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1990 Ubicación: Nivel Nacional Fecha de Publicación: 24/01/2026 Vigente: Según ODPE Salario: S/. 3000.00 Soles mensuales PUESTO: COORDINADOR DISTRITAL NÚMERO: Locación de Servicios NIVEL: Técnicos y Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Pr</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-asistentes-de-oficina-t2.html</t>
+          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-coordinadores-distritales.html</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3416,336 +3351,6 @@
         </is>
       </c>
       <c r="M42" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/ASISTENTE_DE_OFICINA_T2.pdf</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/GUIA_PARA_POSTULAR_ONPE.pdf</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>124</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>ONPE - CONSULTA SI ERES MIEMBRO DE MESA - ELECCIONES GENERALES 2026</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>ONPE</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>El 12 de abril del 2026, es el día de las Elecciones Generales 2026, en ese sentido si deseas conocer si eres miembro de mesa, te informamos que la ONPE ya publicó el link donde puedes CONSULTAR SI ERES MIEMBRO DE MESA , para las Elecciones Generales 2026. Ingresa en el siguiente link para consultar si eres miembro de mesa: http</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>https://www.portaltrabajos.pe/2026/01/onpe-consulta-si-eres-miembro-de-mesa.html</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Portaltrabajo - ONPE</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>126</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>ONPE EG2026: Asistentes Legales</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>ONPE</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Nivel Nacional</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>S/. 4000.00 Soles mensuales</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 126 Ubicación: Nivel Nacional - (Según ODPE Disponible) Fecha de Publicación: 27/01/2026 Vigente: Según ODPE Salario: S/. 4000.00 Soles mensuales PUESTO: ASISTENTES LEGALES NÚMERO: Locación de Servicios NIVEL: Universitarios TIPO DE TRABAJO: Locación de Servicios MO</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-asistentes-legales.html</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-01-27</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Portaltrabajo - ONPE</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/ASISTENTE_LEGAL.pdf</t>
-        </is>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>128</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>ONPE EG2026: (1895) Coordinadores de Centro Poblado</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>ONPE</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Nivel Nacional</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>S/. 3000.00 Soles mensuales</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1895 Ubicación: Nivel Nacional Fecha de Publicación: 24/01/2026 Vigente: Según ODPE Salario: S/. 3000.00 Soles mensuales PUESTO: COORDINADOR DISTRITAL NÚMERO: Locación de Servicios NIVEL: Técnicos y Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Pr</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-coordinadores-de-centro-poblado.html</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-01-24</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Portaltrabajo - ONPE</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/COORDINADOR_DE_CENTRO_%20POBLADO_ODPE_EG2026.pdf</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>129</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>ONPE EG2026: (203) Coordinadores Distritales STAE</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>ONPE</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Lima</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>S/. 3000.00 Soles mensuales</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 203 Ubicación: Lima Fecha de Publicación: 15/02/2026 Vigente: Según ODPE Salario: S/. 3000.00 Soles mensuales PUESTO: COORDINADOR DISTRITAL STAE NÚMERO: Locación de Servicios NIVEL: Técnicos y Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Presenci</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-coordinadores-stae.html</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-01-24</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Portaltrabajo - ONPE</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/COORDINADOR_DISTRITAL_ODPE_STAE_EG2026.pdf</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>https://pe.portaltrabajos.pe/pdf/ONPE/FUNCIONES_COORDINADORES_DISTRITALES_STAE.pdf</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1dbhbM_GVXaUZxEDOVhijNLgx6Nay85em/view?usp=drive_link</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>https://reclutamiento.onpe.gob.pe/login</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>130</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>ONPE EG2026: (1990) Coordinadores Distritales</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>ONPE</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Nivel Nacional</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>S/. 3000.00 Soles mensuales</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Institución: OFICINA NACIONAL DE PROCESOS ELECTORALES Vacantes: 1990 Ubicación: Nivel Nacional Fecha de Publicación: 24/01/2026 Vigente: Según ODPE Salario: S/. 3000.00 Soles mensuales PUESTO: COORDINADOR DISTRITAL NÚMERO: Locación de Servicios NIVEL: Técnicos y Universitarios TIPO DE TRABAJO: Locación de Servicios MODALIDAD: Pr</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>https://www.portaltrabajos.pe/2026/01/onpe-eg2026-coordinadores-distritales.html</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-01-24</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Portaltrabajo - ONPE</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
         <is>
           <t>https://pe.portaltrabajos.pe/pdf/ONPE/COORDINADOR_DISTRITAL_ODPE_EG2026.pdf</t>
         </is>

</xml_diff>